<commit_message>
3 more easy python tasks
ToDo: Testinng
</commit_message>
<xml_diff>
--- a/files/programming-tasks/programmieraufgaben_basicTasks_genByGPT_sven.xlsx
+++ b/files/programming-tasks/programmieraufgaben_basicTasks_genByGPT_sven.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\hefl\files\programming-tasks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7F1188B-6872-4B51-B80B-D76318A671AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{964CE466-926E-4406-98C6-11B2A609F159}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51480" yWindow="-645" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="73">
   <si>
     <t>id</t>
   </si>
@@ -312,12 +312,81 @@
   <si>
     <t>python</t>
   </si>
+  <si>
+    <t>Stell dir vor, du organisierst eine Party mit deinen Freunden und hast mehrere Pizzas bestellt. Um sicherzustellen, dass jeder gleich viele Pizzastücke bekommt, musst du die Gesamtzahl der Pizzastücke durch die Anzahl der Freunde teilen. Deine Aufgabe ist es, eine Funktion teile_pizza zu implementieren, die die Anzahl der Pizzastücke und die Anzahl der Freunde entgegennimmt und die Anzahl der Pizzastücke berechnet, die jeder Freund bekommt. Die Funktion soll die ganzzahlige Anzahl der Pizzastücke pro Person zurückgeben. Wenn es weniger Pizzastücke als Freunde gibt, sollte die Funktion 0 zurückgeben.</t>
+  </si>
+  <si>
+    <t>Pizza teilen</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Stell dir vor, du organisierst eine Party mit deinen Freunden und hast mehrere Pizzas bestellt. Um sicherzustellen, dass jeder gleich viele Pizzastücke bekommt, musst du die Gesamtzahl der Pizzastücke durch die Anzahl der Freunde teilen. Deine Aufgabe ist es, eine Funktion &lt;code&gt;teile_pizza&lt;/code&gt; zu implementieren, die die Anzahl der Pizzastücke und die Anzahl der Freunde entgegennimmt und die Anzahl der Pizzastücke berechnet, die jeder Freund bekommt. Die Funktion soll die ganzzahlige Anzahl der Pizzastücke pro Person zurückgeben. Wenn es weniger Pizzastücke als Freunde gibt, sollte die Funktion 0 zurückgeben.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>import unittest
+class TestTeilePizza(unittest.TestCase):
+    def test_teile_pizza(self):
+        self.assertEqual(teile_pizza(8, 4), 2)
+        self.assertEqual(teile_pizza(10, 0), 0)
+        self.assertEqual(teile_pizza(3, 4), 0)
+if __name__ == "__main__":
+    unittest.main()</t>
+  </si>
+  <si>
+    <t>pizzateilung.py</t>
+  </si>
+  <si>
+    <t>def teile_pizza(pizzastuecke, freunde):
+    # Dein Code hier</t>
+  </si>
+  <si>
+    <t>teile_pizza</t>
+  </si>
+  <si>
+    <t>12, 3</t>
+  </si>
+  <si>
+    <t>Wochenplanung</t>
+  </si>
+  <si>
+    <t>In der Wochenplanung einer Studentenverbindung wird festgelegt, wer an welchem Tag der Woche für das Abendessen zuständig ist. Die Zuweisung der Kochtage erfolgt zyklisch unter den Mitgliedern. Deine Aufgabe besteht darin, eine Funktion assign_cooking_day zu implementieren, die den Namen des für einen bestimmten Tag zuständigen Mitglieds zurückgibt. Die Funktion nimmt zwei Parameter: day_number, die Nummer des Tages, und members, eine Liste der Namen der Mitglieder. Die Zählung beginnt bei Tag 1, der dem ersten Element in der Mitgliederliste entspricht. Nutze den Modulo-Operator, um den entsprechenden Index in der Mitgliederliste zu bestimmen und den Namen des zuständigen Mitglieds zurückzugeben. Dies ist besonders nützlich, um auch für Tage weit in der Zukunft den Koch zuordnen zu können, ohne die Liste manuell erweitern zu müssen.</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;In der Wochenplanung einer Studentenverbindung wird festgelegt, wer an welchem Tag der Woche für das Abendessen zuständig ist. Die Zuweisung der Kochtage erfolgt zyklisch unter den Mitgliedern. Deine Aufgabe besteht darin, eine Funktion &lt;b&gt;assign_cooking_day&lt;/b&gt; zu implementieren, die den Namen des für einen bestimmten Tag zuständigen Mitglieds zurückgibt. Die Funktion nimmt zwei Parameter: &lt;i&gt;day_number&lt;/i&gt;, die Nummer des Tages, und &lt;i&gt;members&lt;/i&gt;, eine Liste der Namen der Mitglieder. Die Zählung beginnt bei Tag 1, der dem ersten Element in der Mitgliederliste entspricht. Nutze den Modulo-Operator, um den entsprechenden Index in der Mitgliederliste zu bestimmen und den Namen des zuständigen Mitglieds zurückzugeben. Dies ist besonders nützlich, um auch für Tage weit in der Zukunft den Koch zuordnen zu können, ohne die Liste manuell erweitern zu müssen.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>cooking_assignment.py</t>
+  </si>
+  <si>
+    <t>import unittest
+from cooking_assignment import assign_cooking_day
+class TestCookingAssignment(unittest.TestCase):
+    def test_assign_cooking_day(self):
+        members = ["Alice", "Bob", "Charlie", "Dana"]
+        self.assertEqual(assign_cooking_day(1, members), "Alice")
+        self.assertEqual(assign_cooking_day(5, members), "Alice")
+        self.assertEqual(assign_cooking_day(7, members), "Charlie")
+if __name__ == "__main__":
+    unittest.main()</t>
+  </si>
+  <si>
+    <t>assign_cooking_day</t>
+  </si>
+  <si>
+    <t>10, ["Alice", "Bob", "Charlie", "Dana"]</t>
+  </si>
+  <si>
+    <t>def assign_cooking_day(day_number, members):
+    # Implementiere hier die Funktion
+# Beispielausführung der Funktion
+if __name__ == "__main__":
+    print(assign_cooking_day(10, ["Alice", "Bob", "Charlie", "Dana"]))</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -397,6 +466,11 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -432,7 +506,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -493,6 +567,17 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="2" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Gut" xfId="1" builtinId="26"/>
@@ -800,8 +885,8 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="28.5" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:N8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="28.5"/>
   <cols>
     <col min="1" max="2" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23.140625" bestFit="1" customWidth="1"/>
@@ -819,7 +904,7 @@
     <col min="15" max="17" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="6" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:14" s="6" customFormat="1" ht="18.75" customHeight="1">
       <c r="A1" s="8" t="s">
         <v>4</v>
       </c>
@@ -861,46 +946,47 @@
       </c>
       <c r="N1" s="13"/>
     </row>
-    <row r="2" spans="1:14" ht="216.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="15">
+    <row r="2" spans="1:14" s="6" customFormat="1" ht="285">
+      <c r="A2" s="25">
         <v>1</v>
       </c>
-      <c r="B2" s="16">
+      <c r="B2" s="26">
         <v>1</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="27" t="s">
         <v>56</v>
       </c>
-      <c r="D2" s="14">
+      <c r="D2" s="27">
         <v>5</v>
       </c>
-      <c r="E2" s="14" t="s">
+      <c r="E2" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="F2" s="14" t="s">
+      <c r="F2" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="G2" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="14" t="s">
+      <c r="H2" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="I2" s="14" t="s">
+      <c r="I2" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="J2" s="14">
+      <c r="J2" s="27">
         <v>0</v>
       </c>
-      <c r="K2" s="14" t="s">
+      <c r="K2" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="L2" s="14" t="s">
+      <c r="L2" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="M2" s="14"/>
-    </row>
-    <row r="3" spans="1:14" ht="114.75" x14ac:dyDescent="0.25">
+      <c r="M2" s="27"/>
+      <c r="N2" s="28"/>
+    </row>
+    <row r="3" spans="1:14" ht="114.75">
       <c r="A3" s="15">
         <v>2</v>
       </c>
@@ -939,7 +1025,7 @@
       </c>
       <c r="M3" s="14"/>
     </row>
-    <row r="4" spans="1:14" ht="153" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" ht="153">
       <c r="A4" s="15">
         <v>3</v>
       </c>
@@ -980,7 +1066,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="178.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" ht="178.5">
       <c r="A5" s="15">
         <v>4</v>
       </c>
@@ -1021,7 +1107,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="191.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" ht="191.25">
       <c r="A6" s="15">
         <v>5</v>
       </c>
@@ -1060,6 +1146,88 @@
       </c>
       <c r="M6" s="14" t="s">
         <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="187.5">
+      <c r="A7" s="1">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1">
+        <v>1</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="D7" s="1">
+        <v>14</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="I7" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="J7" s="1">
+        <v>0</v>
+      </c>
+      <c r="K7" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="M7" s="14" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="225">
+      <c r="A8" s="1">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1">
+        <v>1</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="D8" s="1">
+        <v>14</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="I8" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="J8" s="1">
+        <v>0</v>
+      </c>
+      <c r="K8" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="M8" s="14" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -1074,14 +1242,14 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:D62"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="60" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="60" customHeight="1"/>
   <cols>
     <col min="1" max="2" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="129.7109375" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="60" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1095,7 +1263,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="60" customHeight="1">
       <c r="A2" s="15">
         <v>1</v>
       </c>
@@ -1109,7 +1277,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" ht="60" customHeight="1">
       <c r="A3" s="15">
         <v>2</v>
       </c>
@@ -1123,7 +1291,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" ht="60" customHeight="1">
       <c r="A4" s="15">
         <v>3</v>
       </c>
@@ -1137,7 +1305,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" ht="60" customHeight="1">
       <c r="A5" s="15">
         <v>4</v>
       </c>
@@ -1151,7 +1319,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" ht="60" customHeight="1">
       <c r="A6" s="15">
         <v>5</v>
       </c>
@@ -1165,277 +1333,297 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-    </row>
-    <row r="8" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-    </row>
-    <row r="9" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" ht="60" customHeight="1">
+      <c r="A7" s="3">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3">
+        <v>6</v>
+      </c>
+      <c r="C7" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="60" customHeight="1">
+      <c r="A8" s="3">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3">
+        <v>7</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="60" customHeight="1">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="D9" s="4"/>
     </row>
-    <row r="10" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" ht="60" customHeight="1">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="D10" s="4"/>
     </row>
-    <row r="11" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" ht="60" customHeight="1">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="D11" s="4"/>
     </row>
-    <row r="12" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" ht="60" customHeight="1">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="D12" s="4"/>
     </row>
-    <row r="13" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" ht="60" customHeight="1">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="D13" s="4"/>
     </row>
-    <row r="14" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" ht="60" customHeight="1">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="D14" s="4"/>
     </row>
-    <row r="15" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" ht="60" customHeight="1">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="D15" s="4"/>
     </row>
-    <row r="16" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" ht="60" customHeight="1">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="D16" s="4"/>
     </row>
-    <row r="17" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" ht="60" customHeight="1">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="D17" s="4"/>
     </row>
-    <row r="18" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" ht="60" customHeight="1">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="D18" s="4"/>
     </row>
-    <row r="19" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" ht="60" customHeight="1">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="D19" s="4"/>
     </row>
-    <row r="20" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" ht="60" customHeight="1">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="D20" s="4"/>
     </row>
-    <row r="21" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" ht="60" customHeight="1">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="D21" s="4"/>
     </row>
-    <row r="22" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" ht="60" customHeight="1">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="D22" s="4"/>
     </row>
-    <row r="23" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" ht="60" customHeight="1">
       <c r="A23" s="3"/>
       <c r="B23" s="3"/>
       <c r="D23" s="4"/>
     </row>
-    <row r="24" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" ht="60" customHeight="1">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="D24" s="4"/>
     </row>
-    <row r="25" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" ht="60" customHeight="1">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
       <c r="D25" s="4"/>
     </row>
-    <row r="26" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" ht="60" customHeight="1">
       <c r="A26" s="3"/>
       <c r="B26" s="3"/>
       <c r="D26" s="4"/>
     </row>
-    <row r="27" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" ht="60" customHeight="1">
       <c r="A27" s="3"/>
       <c r="B27" s="3"/>
       <c r="D27" s="4"/>
     </row>
-    <row r="28" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" ht="60" customHeight="1">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
       <c r="D28" s="4"/>
     </row>
-    <row r="29" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" ht="60" customHeight="1">
       <c r="A29" s="3"/>
       <c r="B29" s="3"/>
       <c r="D29" s="4"/>
     </row>
-    <row r="30" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" ht="60" customHeight="1">
       <c r="A30" s="3"/>
       <c r="B30" s="3"/>
       <c r="D30" s="4"/>
     </row>
-    <row r="31" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" ht="60" customHeight="1">
       <c r="A31" s="3"/>
       <c r="B31" s="3"/>
       <c r="D31" s="4"/>
     </row>
-    <row r="32" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" ht="60" customHeight="1">
       <c r="A32" s="3"/>
       <c r="B32" s="3"/>
       <c r="D32" s="4"/>
     </row>
-    <row r="33" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" ht="60" customHeight="1">
       <c r="A33" s="3"/>
       <c r="B33" s="3"/>
       <c r="D33" s="4"/>
     </row>
-    <row r="34" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" ht="60" customHeight="1">
       <c r="A34" s="3"/>
       <c r="B34" s="3"/>
       <c r="D34" s="4"/>
     </row>
-    <row r="35" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" ht="60" customHeight="1">
       <c r="A35" s="3"/>
       <c r="B35" s="3"/>
       <c r="D35" s="5"/>
     </row>
-    <row r="36" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" ht="60" customHeight="1">
       <c r="A36" s="3"/>
       <c r="B36" s="3"/>
       <c r="D36" s="5"/>
     </row>
-    <row r="37" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" ht="60" customHeight="1">
       <c r="A37" s="3"/>
       <c r="B37" s="3"/>
       <c r="D37" s="5"/>
     </row>
-    <row r="38" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" ht="60" customHeight="1">
       <c r="A38" s="3"/>
       <c r="B38" s="3"/>
       <c r="D38" s="5"/>
     </row>
-    <row r="39" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" ht="60" customHeight="1">
       <c r="A39" s="3"/>
       <c r="B39" s="3"/>
       <c r="D39" s="5"/>
     </row>
-    <row r="40" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" ht="60" customHeight="1">
       <c r="A40" s="3"/>
       <c r="B40" s="3"/>
       <c r="D40" s="5"/>
     </row>
-    <row r="41" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" ht="60" customHeight="1">
       <c r="A41" s="3"/>
       <c r="B41" s="3"/>
       <c r="D41" s="5"/>
     </row>
-    <row r="42" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" ht="60" customHeight="1">
       <c r="A42" s="3"/>
       <c r="B42" s="3"/>
       <c r="D42" s="5"/>
     </row>
-    <row r="43" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" ht="60" customHeight="1">
       <c r="A43" s="3"/>
       <c r="B43" s="3"/>
       <c r="D43" s="5"/>
     </row>
-    <row r="44" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" ht="60" customHeight="1">
       <c r="A44" s="3"/>
       <c r="B44" s="3"/>
       <c r="D44" s="5"/>
     </row>
-    <row r="45" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" ht="60" customHeight="1">
       <c r="A45" s="3"/>
       <c r="B45" s="3"/>
       <c r="D45" s="5"/>
     </row>
-    <row r="46" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" ht="60" customHeight="1">
       <c r="A46" s="3"/>
       <c r="B46" s="3"/>
       <c r="D46" s="5"/>
     </row>
-    <row r="47" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" ht="60" customHeight="1">
       <c r="A47" s="3"/>
       <c r="B47" s="3"/>
       <c r="D47" s="5"/>
     </row>
-    <row r="48" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" ht="60" customHeight="1">
       <c r="A48" s="3"/>
       <c r="B48" s="3"/>
       <c r="D48" s="5"/>
     </row>
-    <row r="49" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" ht="60" customHeight="1">
       <c r="A49" s="3"/>
       <c r="B49" s="3"/>
       <c r="D49" s="5"/>
     </row>
-    <row r="50" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" ht="60" customHeight="1">
       <c r="A50" s="3"/>
       <c r="B50" s="3"/>
       <c r="D50" s="5"/>
     </row>
-    <row r="51" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" ht="60" customHeight="1">
       <c r="A51" s="3"/>
       <c r="B51" s="3"/>
       <c r="D51" s="5"/>
     </row>
-    <row r="52" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" ht="60" customHeight="1">
       <c r="A52" s="3"/>
       <c r="B52" s="3"/>
       <c r="D52" s="5"/>
     </row>
-    <row r="53" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" ht="60" customHeight="1">
       <c r="A53" s="3"/>
       <c r="B53" s="3"/>
       <c r="D53" s="5"/>
     </row>
-    <row r="54" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" ht="60" customHeight="1">
       <c r="A54" s="3"/>
       <c r="B54" s="3"/>
       <c r="D54" s="5"/>
     </row>
-    <row r="55" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" ht="60" customHeight="1">
       <c r="A55" s="3"/>
       <c r="B55" s="3"/>
     </row>
-    <row r="56" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" ht="60" customHeight="1">
       <c r="A56" s="3"/>
       <c r="B56" s="3"/>
     </row>
-    <row r="57" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" ht="60" customHeight="1">
       <c r="A57" s="3"/>
       <c r="B57" s="3"/>
     </row>
-    <row r="58" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" ht="60" customHeight="1">
       <c r="A58" s="3"/>
       <c r="B58" s="3"/>
     </row>
-    <row r="59" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" ht="60" customHeight="1">
       <c r="A59" s="3"/>
       <c r="B59" s="3"/>
       <c r="D59" s="5"/>
     </row>
-    <row r="60" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" ht="60" customHeight="1">
       <c r="A60" s="3"/>
       <c r="B60" s="3"/>
       <c r="D60" s="5"/>
     </row>
-    <row r="61" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" ht="60" customHeight="1">
       <c r="A61" s="3"/>
       <c r="B61" s="3"/>
       <c r="C61" s="5"/>
       <c r="D61" s="5"/>
     </row>
-    <row r="62" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" ht="60" customHeight="1">
       <c r="A62" s="3"/>
       <c r="B62" s="3"/>
       <c r="D62" s="5"/>

</xml_diff>

<commit_message>
cpp-support-codingTaskEditor small fix and cpp example task
</commit_message>
<xml_diff>
--- a/files/programming-tasks/programmieraufgaben_basicTasks_genByGPT_sven.xlsx
+++ b/files/programming-tasks/programmieraufgaben_basicTasks_genByGPT_sven.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\hefl\files\programming-tasks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B57907BD-E52C-4A67-AACA-409FF9A4922A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1E154C4-3E70-42C4-89D7-B90042A776DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51480" yWindow="-645" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aufgaben" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="78">
   <si>
     <t>id</t>
   </si>
@@ -91,26 +91,6 @@
   </si>
   <si>
     <t>Hallo Welt</t>
-  </si>
-  <si>
-    <t>Erweitere das vorhandene Python-Programm so, dass die Funktion wilkommen() statt „Hallo“ nun „Hallo Welt“ ausgibt.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    &lt;h1&gt;Eure erste Aufgabe:&lt;/h1&gt;
-    &lt;p&gt;Erweitere das vorhandene Python-Programm so, dass die Funktion wilkommen() statt „Hallo“ nun „Hallo Welt“ ausgibt.&lt;/p&gt;
-    &lt;h2&gt;Hinweise zu Programmieraufgaben:&lt;/h2&gt;
-    &lt;h3&gt;Ausführen und Testen:&lt;/h3&gt;
-    &lt;p&gt;Keine Sorge, ihr müsst nicht selbst überprüfen, ob euer Code korrekt funktioniert. Unser System übernimmt das automatisch für euch. Wenn alles passt, seht ihr eine Punktzahl von 100/100. Das ist euer Ziel!&lt;/p&gt;
-    &lt;h3&gt;Feedback:&lt;/h3&gt;
-    &lt;p&gt;Falls ihr mal nicht weiterwisst, steht euch unser Tutor Kai mit Rat und Tat zur Seite. Nachdem ihr euren Code zum ersten Mal ausgeführt habt, werdet ihr zwei Feedback-Buttons sehen, die euch helfen können. Da wir das Feedback-System noch verbessern möchten, würden wir uns freuen, wenn ihr nach der Nutzung eine Bewertung zwischen 1 und 7 Sternen abgebt. Ihr könnt auch gerne zusätzliche Kommentare hinterlassen, falls ihr spezielle Anregungen oder Wünsche habt.&lt;/p&gt;
-    &lt;p&gt;Wir wünschen euch viel Erfolg und Spaß bei dieser ersten Herausforderung!&lt;/p&gt;
-    &lt;p&gt;Euer &lt;strong&gt;GOALS -Team&lt;/strong&gt;&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>halloWelt.py</t>
-  </si>
-  <si>
-    <t>willkommen</t>
   </si>
   <si>
     <t>Python Variabeln</t>
@@ -203,11 +183,6 @@
   <si>
     <t>def convert_to_number(s):
     # Implementiere die Funktion hier</t>
-  </si>
-  <si>
-    <t>def willkommen():
-    return "Hallo" # Passen Sie diese Zeile an.
-print(willkommen())</t>
   </si>
   <si>
     <t>python</t>
@@ -279,16 +254,6 @@
   </si>
   <si>
     <t>In dieser Übung geht es darum, die Grundlagen von Variablen in Python zu verstehen und anzuwenden. Deine Aufgabe ist es, eine Funktion namens initialisiere_variable zu implementieren, die eine Variable namens meine_variable deklariert und mit dem Wert 100 initialisiert. Die Funktion sollte dann diese Variable zurückgeben.</t>
-  </si>
-  <si>
-    <t>import unittest
-from halloWelt import willkommen
-class TestWillkommen(unittest.TestCase):
-    def test_willkommen(self):
-        self.assertEqual(willkommen(), "Hallo Welt")
-# Dies führt die Tests aus, wenn das Skript direkt ausgeführt wird.
-if __name__ == '__main__':
-    unittest.main()</t>
   </si>
   <si>
     <t>import unittest
@@ -348,6 +313,83 @@
         self.assertEqual(teile_pizza(3, 4), 0)
 if __name__ == "__main__":
     unittest.main()</t>
+  </si>
+  <si>
+    <t>CPP TEST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    &lt;h1&gt;CPP Test&lt;/h1&gt;
+</t>
+  </si>
+  <si>
+    <t>main.cpp</t>
+  </si>
+  <si>
+    <t>testFile</t>
+  </si>
+  <si>
+    <t>#define DOCTEST_CONFIG_IMPLEMENT_WITH_MAIN
+#include &lt;JsonReporter.h&gt;
+#include "Calculator.h"
+#include "Greeter.h"
+TEST_CASE("Calculator add method") {
+    Calculator calc;
+    SUBCASE("Adding positive numbers") {
+        REQUIRE(calc.add(5, 3) == 8);
+    }
+    SUBCASE("Adding negative numbers") {
+        REQUIRE(calc.add(-2, -4) == -6);
+    }
+}
+TEST_CASE("Greeter greet method") {
+    Greeter greeter;
+    SUBCASE("Greeting a person") {
+        REQUIRE(greeter.greet("John") == "Hello, John!");
+    }
+    SUBCASE("Greeting an empty string") {
+        REQUIRE(greeter.greet("") == "Hello, !");
+    }
+}</t>
+  </si>
+  <si>
+    <t>#include &lt;iostream&gt;
+#include "Calculator.h"
+#include "Greeter.h"
+int main() {
+    Calculator calc;
+    Greeter greeter;
+    int sum = calc.add(5, 3);
+    std::cout &lt;&lt; "Sum of 5 and 3 is: " &lt;&lt; sum &lt;&lt; std::endl;
+    std::string greeting = greeter.greet("World");
+    std::cout &lt;&lt; greeting &lt;&lt; std::endl;
+    return 0;
+}</t>
+  </si>
+  <si>
+    <t>Calculator.h</t>
+  </si>
+  <si>
+    <t>class Calculator {
+public:
+    int add(int a, int b) {
+        return a + b;
+    }
+};</t>
+  </si>
+  <si>
+    <t>Greeter.h</t>
+  </si>
+  <si>
+    <t>#include &lt;string&gt;
+class Greeter {
+public:
+    std::string greet(const std::string&amp; name) {
+        return "Hello, " + name + "!";
+    }
+};</t>
+  </si>
+  <si>
+    <t>cpp</t>
   </si>
 </sst>
 </file>
@@ -911,7 +953,7 @@
       </c>
       <c r="N1" s="13"/>
     </row>
-    <row r="2" spans="1:14" s="6" customFormat="1" ht="285">
+    <row r="2" spans="1:14" s="6" customFormat="1" ht="409.5">
       <c r="A2" s="22">
         <v>1</v>
       </c>
@@ -919,7 +961,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="24" t="s">
-        <v>48</v>
+        <v>77</v>
       </c>
       <c r="D2" s="24">
         <v>5</v>
@@ -928,26 +970,24 @@
         <v>18</v>
       </c>
       <c r="F2" s="24" t="s">
-        <v>19</v>
+        <v>67</v>
       </c>
       <c r="G2" s="24" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="H2" s="24" t="s">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="I2" s="24" t="s">
-        <v>21</v>
+        <v>69</v>
       </c>
       <c r="J2" s="24">
         <v>0</v>
       </c>
       <c r="K2" s="24" t="s">
-        <v>16</v>
-      </c>
-      <c r="L2" s="24" t="s">
-        <v>22</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="L2" s="24"/>
       <c r="M2" s="24"/>
       <c r="N2" s="25"/>
     </row>
@@ -959,25 +999,25 @@
         <v>1</v>
       </c>
       <c r="C3" s="25" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="D3" s="25">
         <v>6</v>
       </c>
       <c r="E3" s="25" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F3" s="25" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="G3" s="26" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="H3" s="25" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="I3" s="25" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="J3" s="25">
         <v>0</v>
@@ -986,7 +1026,7 @@
         <v>16</v>
       </c>
       <c r="L3" s="25" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:14" s="6" customFormat="1" ht="195">
@@ -997,25 +1037,25 @@
         <v>1</v>
       </c>
       <c r="C4" s="24" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="D4" s="24">
         <v>7</v>
       </c>
       <c r="E4" s="24" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F4" s="25" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G4" s="24" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="H4" s="24" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="J4" s="24">
         <v>0</v>
@@ -1024,10 +1064,10 @@
         <v>16</v>
       </c>
       <c r="L4" s="27" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="M4" s="27" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="N4" s="25"/>
     </row>
@@ -1039,25 +1079,25 @@
         <v>1</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="D5" s="24">
         <v>17</v>
       </c>
       <c r="E5" s="24" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F5" s="25" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="G5" s="24" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="H5" s="24" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="I5" s="25" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="J5" s="24">
         <v>0</v>
@@ -1066,10 +1106,10 @@
         <v>16</v>
       </c>
       <c r="L5" s="27" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="M5" s="24" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="N5" s="25"/>
     </row>
@@ -1081,25 +1121,25 @@
         <v>1</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="D6" s="24">
         <v>15</v>
       </c>
       <c r="E6" s="24" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="G6" s="24" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="H6" s="24" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="I6" s="24" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="J6" s="24">
         <v>0</v>
@@ -1108,10 +1148,10 @@
         <v>16</v>
       </c>
       <c r="L6" s="24" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="M6" s="24" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="N6" s="25"/>
     </row>
@@ -1123,25 +1163,25 @@
         <v>1</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="D7" s="8">
         <v>14</v>
       </c>
       <c r="E7" s="24" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="I7" s="24" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="J7" s="8">
         <v>0</v>
@@ -1150,10 +1190,10 @@
         <v>16</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="M7" s="24" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="N7" s="25"/>
     </row>
@@ -1165,25 +1205,25 @@
         <v>1</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="D8" s="8">
         <v>14</v>
       </c>
       <c r="E8" s="24" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="I8" s="24" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="J8" s="8">
         <v>0</v>
@@ -1192,10 +1232,10 @@
         <v>16</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="M8" s="24" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="N8" s="25"/>
     </row>
@@ -1240,10 +1280,10 @@
         <v>1</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>21</v>
+        <v>69</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>47</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="60" customHeight="1">
@@ -1254,10 +1294,10 @@
         <v>2</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D3" s="20" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="60" customHeight="1">
@@ -1268,10 +1308,10 @@
         <v>3</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="60" customHeight="1">
@@ -1282,10 +1322,10 @@
         <v>4</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="60" customHeight="1">
@@ -1296,10 +1336,10 @@
         <v>5</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="60" customHeight="1">
@@ -1310,10 +1350,10 @@
         <v>6</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="60" customHeight="1">
@@ -1324,21 +1364,39 @@
         <v>7</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="60" customHeight="1">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="D9" s="4"/>
+      <c r="A9" s="3">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3">
+        <v>1</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="10" spans="1:4" ht="60" customHeight="1">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="D10" s="4"/>
+      <c r="A10" s="3">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3">
+        <v>1</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="11" spans="1:4" ht="60" customHeight="1">
       <c r="A11" s="3"/>

</xml_diff>